<commit_message>
Fixed Compare menu and Validate menu
</commit_message>
<xml_diff>
--- a/MenuComparison.xlsx
+++ b/MenuComparison.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="Menu Comparison" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Menu Comparison'!$E$1:$E$367</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -915,18 +918,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1369,28 +1372,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1514,8 +1517,9 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1902,7 +1906,10 @@
   <dimension ref="A1:E367"/>
   <sheetFormatPr defaultColWidth="7.94117647058824" defaultRowHeight="17.6" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="5" width="31.9852941176471" customWidth="1"/>
+    <col min="1" max="2" width="31.9852941176471" customWidth="1"/>
+    <col min="3" max="3" width="48.6544117647059" customWidth="1"/>
+    <col min="4" max="4" width="42.2794117647059" customWidth="1"/>
+    <col min="5" max="5" width="31.9852941176471" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2000,7 +2007,7 @@
       <c r="C6" t="s">
         <v>16</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E6" t="s">
@@ -8145,10 +8152,16 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="E1:E367" etc:filterBottomFollowUsedRange="0">
+    <extLst/>
+  </autoFilter>
+  <hyperlinks>
+    <hyperlink ref="D6" r:id="rId1" display="https://dev-suny-geneseo.pantheonsite.io/wp-content/uploads/2025/11/ReferenceLetterForm.pdf"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E367" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E5 A6:C6 E6 A7:E9 A10:C10 E10 A11:E367" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>